<commit_message>
Created first C3DC testcase which needs fix for 2 tabs
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\epishinavv\git\Commons_Automation\InputFiles\C3DC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sohilz2/Automation/Commons_Automation/InputFiles/C3DC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD10B4C-10BD-48F0-BFFC-471E18AAED9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE55A0D-FF20-E746-9644-7F8F7F5039F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35070" yWindow="1320" windowWidth="14250" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-41060" yWindow="1300" windowWidth="35920" windowHeight="22300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,84 +40,12 @@
     <t>StudiesTab</t>
   </si>
   <si>
-    <t>SELECT DISTINCT
-     std.dbgap_accession AS "dbGaP Accession",
-     std.study_name AS "Study Name"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE  
-    std.dbgap_accession = 'phs000463' AND prt.sex_at_birth = 'Female';</t>
-  </si>
-  <si>
-    <t>SELECT 
-    COUNT(DISTINCT dgn.diagnosis) AS Diagnoses,
-    COUNT(DISTINCT prt.participant_id) AS Participants,
-    COUNT(DISTINCT std.study_id) AS Studies
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE     
-    std.dbgap_accession = 'phs000463' AND prt.sex_at_birth = 'Female';</t>
-  </si>
-  <si>
-    <t>TC01_C3DC_phs000463_SexAtBirth-Female_TSVData.xlsx</t>
-  </si>
-  <si>
     <t>TC01_C3DC_phs000463_SexAtBirth-Female_WebData.xlsx</t>
   </si>
   <si>
     <t>ParticipantsTab</t>
   </si>
   <si>
-    <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    REPLACE(prt.race, ';', ', ') AS "Race",
-    prt.sex_at_birth AS "Sex at Birth",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000463' AND prt.sex_at_birth = 'Female'
-ORDER BY 
-    prt.participant_id ASC
-LIMIT 100;</t>
-  </si>
-  <si>
     <t>DiagnosisTab</t>
   </si>
   <si>
@@ -128,41 +56,6 @@
   </si>
   <si>
     <t>SurvivalTab</t>
-  </si>
-  <si>
-    <t>SELECT DISTINCT
-    prt.participant_id AS "Participant Id",
-    dgn.diagnosis_id AS "Diagnosis Id",
-    dgn.diagnosis AS "Diagnosis",
-    CASE 
-    WHEN dgn.age_at_diagnosis = -999 THEN 'Not Reported'
-    WHEN dgn.age_at_diagnosis &gt;= 1000 THEN 
-        substr(dgn.age_at_diagnosis, 1, length(dgn.age_at_diagnosis) - 3) || ',' || substr(dgn.age_at_diagnosis, -3)
-    ELSE 
-        dgn.age_at_diagnosis 
-END AS "Age at Diagnosis (days)",
-    dgn.anatomic_site AS "Anatomic Site",
-    dgn.diagnosis_classification_system AS "Diagnosis Classification System",
-    std.dbgap_accession AS "dbGaP Accession"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt ON 1=1
-LEFT JOIN 
-    df_diagnoses dgn ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs000463' AND prt.sex_at_birth = 'Female' AND dgn.diagnosis_id IS NOT NULL
-ORDER BY 
-    prt.participant_id ASC
-LIMIT 100;</t>
   </si>
   <si>
     <t>GeneticAnalysisTab</t>
@@ -305,14 +198,123 @@
    srv.survival_id ASC
 LIMIT 100;</t>
   </si>
+  <si>
+    <t>TC01_C3DC_phs000463_SexAtBirth-Female_DbData.xlsx</t>
+  </si>
+  <si>
+    <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000463'
+  AND p.sex_at_birth = 'Female'
+OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
+OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
+OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
+RETURN count(DISTINCT s) AS studies,
+       count(DISTINCT p) AS participants,
+       count(DISTINCT sm) AS samples,
+       count(DISTINCT f) + count(DISTINCT fp) AS files</t>
+  </si>
+  <si>
+    <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000463'
+  AND p.sex_at_birth = 'Female'
+RETURN p.participant_id AS participant_id,
+       s.study_id AS study_id,
+       p.sex_at_birth AS sex_at_birth,
+       reduce(text = '', value IN coalesce(p.race, []) | CASE WHEN text = '' THEN value ELSE text + '; ' + value END) AS race
+ORDER BY p.participant_id
+LIMIT 100;</t>
+  </si>
+  <si>
+    <t>MATCH (s:study)
+WHERE EXISTS {
+  MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+  WHERE s.dbgap_accession = 'phs000463' AND p.sex_at_birth = 'Female'
+}
+WITH s
+MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, count(DISTINCT sp) AS num_of_participants
+OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
+OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
+ORDER BY diagnosis_n DESC, diagnosis_name
+WITH s, num_of_participants, num_of_samples,
+     [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL][0..5] AS diagnosis_items
+OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+UNWIND CASE WHEN d2 IS NULL THEN [null] ELSE coalesce(d2.anatomic_site, [null]) END AS site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site, count(DISTINCT dp2) AS site_n
+ORDER BY site_n DESC, site
+WITH s, num_of_participants, num_of_samples, diagnosis_items,
+     [item IN collect(CASE WHEN site IS NULL THEN null ELSE site + ' (' + toString(site_n) + ')' END) WHERE item IS NOT NULL][0..5] AS site_items
+OPTIONAL MATCH (f)-[:of_clinical_measure_file|of_generic_file]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site_items, f.file_type AS file_type, count(f) AS type_n
+ORDER BY type_n DESC, file_type
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site_items,
+     sum(CASE WHEN file_type IS NULL THEN 0 ELSE type_n END) AS num_of_files,
+     [item IN collect(CASE WHEN file_type IS NULL THEN null ELSE file_type + ' (' + toString(type_n) + ')' END) WHERE item IS NOT NULL][0..5] AS file_type_items
+OPTIONAL MATCH (pub:publication)-[:of_publication]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site_items, num_of_files, file_type_items,
+     [id IN collect(pub.pubmed_id) WHERE id IS NOT NULL] AS pubmed_ids
+OPTIONAL MATCH (per:study_personnel)-[:of_study_personnel]-&gt;(s)
+WHERE per IS NULL OR per.personnel_type = 'PI'
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site_items, num_of_files, file_type_items, pubmed_ids,
+     [name IN collect(per.personnel_name) WHERE name IS NOT NULL] AS investigators
+OPTIONAL MATCH (fund:study_funding)-[:of_study_funding]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, site_items, num_of_files, file_type_items, pubmed_ids, investigators,
+     [id IN collect(fund.grant_id) WHERE id IS NOT NULL] AS grant_ids
+RETURN s.study_name AS study_name,
+       s.study_id AS study_id,
+       s.study_phase AS study_phase,
+       reduce(text = '', item IN diagnosis_items | CASE WHEN text = '' THEN item ELSE text + '\n' + item END) AS diagnosis,
+       reduce(text = '', item IN site_items | CASE WHEN text = '' THEN item ELSE text + '\n' + item END) AS anatomic_site,
+       toString(num_of_participants) AS num_of_participants,
+       toString(num_of_samples) AS num_of_samples,
+       toString(num_of_files) AS num_of_files,
+       reduce(text = '', item IN file_type_items | CASE WHEN text = '' THEN item ELSE text + '\n' + item END) AS file_type,
+       reduce(text = '', item IN pubmed_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS pubmed_id,
+       reduce(text = '', item IN investigators | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS personnel_name,
+       reduce(text = '', item IN grant_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS grant_id
+ORDER BY s.study_name
+LIMIT 100;</t>
+  </si>
+  <si>
+    <t>MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000463' AND p.sex_at_birth = 'Female'
+RETURN p.participant_id AS participant_id,
+       d.diagnosis_id AS diagnosis_id,
+       d.diagnosis AS diagnosis,
+       CASE
+         WHEN d.age_at_diagnosis IS NULL OR d.age_at_diagnosis = -999 THEN 'Not Reported'
+         ELSE toString(d.age_at_diagnosis)
+       END AS age_at_diagnosis,
+       reduce(text = '', value IN coalesce(d.anatomic_site, []) | CASE WHEN text = '' THEN value ELSE text + ', ' + value END) AS anatomic_site,
+       reduce(text = '', value IN coalesce(d.diagnosis_classification_system, []) | CASE WHEN text = '' THEN value ELSE text + ', ' + value END) AS diagnosis_classification_system,
+       s.dbgap_accession AS dbgap_accession
+ORDER BY p.participant_id
+LIMIT 100;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -366,11 +368,17 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -698,16 +706,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="75.77734375" customWidth="1"/>
-    <col min="3" max="3" width="60.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="75.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -724,81 +732,80 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="297" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="297" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="372" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="333" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B4" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="372" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C10" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Files tab query to every testcase
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
@@ -16,12 +16,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -72,11 +79,14 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -509,7 +519,7 @@
           <t>ParticipantsTab</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000463'
@@ -567,7 +577,7 @@
 WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
 OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
 WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
-ORDER BY diagnosis_n DESC, diagnosis_name
+ORDER BY diagnosis_n DESC, diagnosis_name DESC
 WITH s, num_of_participants, num_of_samples,
      [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL] AS diagnosis_all
 WITH s, num_of_participants, num_of_samples,
@@ -575,32 +585,18 @@
      size(diagnosis_all) &gt; 5 AS diagnosis_more
 OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
 UNWIND CASE WHEN d2 IS NULL THEN [null] ELSE coalesce(d2.anatomic_site, [null]) END AS site
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT dp2) AS site_n
-ORDER BY site_n DESC, site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT d2) AS site_n
+ORDER BY site_n DESC, site DESC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      [item IN collect(CASE WHEN site IS NULL THEN null ELSE site + ' (' + toString(site_n) + ')' END) WHERE item IS NOT NULL] AS site_all
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      site_all[0..5] AS site_items,
      size(site_all) &gt; 5 AS site_more
-OPTIONAL MATCH (sf)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file]-&gt;(:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+OPTIONAL MATCH (s)&lt;-[*..6]-(fl)
+WHERE (fl:clinical_measure_file OR fl:generic_file OR fl:sequencing_file OR fl:pathology_file OR fl:radiology_file OR fl:methylation_array_file OR fl:cytogenomic_file)
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
-     sf.file_type AS file_type, count(DISTINCT sf) AS type_n
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
-     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS sample_file_types
-OPTIONAL MATCH (pf)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
-     pf.file_type AS file_type, count(DISTINCT pf) AS type_n
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
-     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS participant_file_types
-OPTIONAL MATCH (stf)-[:of_clinical_measure_file|of_generic_file]-&gt;(s)
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types, participant_file_types,
-     stf.file_type AS file_type, count(DISTINCT stf) AS type_n
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
-     sample_file_types + participant_file_types + [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS file_types
-UNWIND CASE WHEN size(file_types) = 0 THEN [{t: null, n: 0}] ELSE file_types END AS ft
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
-     ft.t AS file_type, sum(ft.n) AS type_n
-ORDER BY type_n DESC, file_type
+     fl.file_type AS file_type, count(DISTINCT fl.dcf_indexd_guid) AS type_n
+ORDER BY type_n DESC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
      sum(CASE WHEN file_type IS NULL THEN 0 ELSE type_n END) AS num_of_files,
      [item IN collect(CASE WHEN file_type IS NULL THEN null ELSE file_type + ' (' + toString(type_n) + ')' END) WHERE item IS NOT NULL] AS file_type_all
@@ -706,7 +702,7 @@
   MATCH (t:treatment_chemotherapy)-[:of_treatment_chemotherapy]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
   WHERE s.dbgap_accession = 'phs002883' AND p.sex_at_birth = 'Female'
   RETURN p.participant_id AS participant_id,
-         t.guid AS treatment_id,
+         t.treatment_chemotherapy_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
          reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
@@ -716,7 +712,7 @@
   MATCH (t:treatment_radiation)-[:of_treatment_radiation]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
   WHERE s.dbgap_accession = 'phs000463' AND p.sex_at_birth = 'Female'
   RETURN p.participant_id AS participant_id,
-         t.guid AS treatment_id,
+         t.treatment_radiation_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
          reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
@@ -726,7 +722,7 @@
   MATCH (t:treatment_surgery)-[:of_treatment_surgery]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
   WHERE s.dbgap_accession = 'phs002883' AND p.sex_at_birth = 'Female'
   RETURN p.participant_id AS participant_id,
-         t.guid AS treatment_id,
+         t.treatment_surgery_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
          reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
@@ -736,7 +732,7 @@
   MATCH (t:treatment_other)-[:of_treatment_other]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
   WHERE s.dbgap_accession = 'phs002883' AND p.sex_at_birth = 'Female'
   RETURN p.participant_id AS participant_id,
-         t.guid AS treatment_id,
+         t.treatment_other_id AS treatment_id,
          CASE WHEN t.age_at_treatment_start IS NULL OR t.age_at_treatment_start = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_start) END AS age_start,
          CASE WHEN t.age_at_treatment_end IS NULL OR t.age_at_treatment_end = -999 THEN 'Not Reported' ELSE toString(t.age_at_treatment_end) END AS age_end,
          reduce(text = '', item IN coalesce(t.treatment_type, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS treatment_type,
@@ -833,7 +829,36 @@
       </c>
       <c r="C9" s="1" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="395" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FilesTab</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000463'
+  AND p.sex_at_birth = 'Female'
+MATCH (sm:sample)-[:of_sample]-&gt;(p)
+MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
+RETURN f.file_name AS `File Name`,
+       reduce(text = '', item IN coalesce(f.data_category, []) | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Data Category`,
+       f.file_type AS `File Type`,
+       s.dbgap_accession AS `Study ID`,
+       p.participant_id AS `Participant ID`,
+       sm.sample_id AS `Sample ID`,
+       reduce(text = '', site IN coalesce(sm.anatomic_site, []) | CASE WHEN text = '' THEN site ELSE text + ';' + site END) AS `Anatomic Site`,
+       CASE
+         WHEN sm.participant_age_at_collection IS NULL OR sm.participant_age_at_collection = -999 THEN 'Not Reported'
+         ELSE toString(sm.participant_age_at_collection)
+       END AS `Age at Collection`,
+       sm.sample_tumor_status AS `Sample Tumor Status`,
+       sm.tumor_spatial_extent AS `Tumor Spatial Extent`
+ORDER BY f.file_name
+LIMIT 100;</t>
+        </is>
+      </c>
       <c r="C10" s="1" t="n"/>
     </row>
   </sheetData>

</xml_diff>